<commit_message>
Set packhouse crew to 20-30 workers (25 used) in simple model
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UfRpkuKRMFz5PChZk64pJu
</commit_message>
<xml_diff>
--- a/Banana_Packhouse_Simple_Model.xlsx
+++ b/Banana_Packhouse_Simple_Model.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="190">
   <si>
     <t xml:space="preserve">Banana Packhouse &amp; Cooling – Unit Economics (Sitpur, Vadodara)</t>
   </si>
@@ -125,6 +125,24 @@
     <t xml:space="preserve">Cost of production for premium banana is about ₹11/kg.</t>
   </si>
   <si>
+    <t xml:space="preserve">Packhouse workers per day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">workers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">De-handing, washing, grading and packing crew for 36 t a day (loaders and cleaners are counted separately).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Packhouse worker wage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">₹/day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gujarat minimum wage for unskilled workers (Apr–Sep 2026).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Our edge vs traditional handling, per kg sold</t>
   </si>
   <si>
@@ -182,7 +200,7 @@
     <t xml:space="preserve">Packhouse labour (de-handing, washing, grading, packing)</t>
   </si>
   <si>
-    <t xml:space="preserve">~30–50 workers at Gujarat minimum wage (₹512/day) for 38 t a day. Scale brings this below the ₹1.50 in your first draft (which assumed 13 t a day).</t>
+    <t xml:space="preserve">20 / 25 / 30 workers × ₹512.50 a day ÷ 36,000 kg sold a day. Scale brings this well below the ₹1.50 in your first draft (which assumed 13 t a day).</t>
   </si>
   <si>
     <t xml:space="preserve">Post-harvest treatment (alum wash + fungicide dip + wash water)</t>
@@ -554,7 +572,7 @@
     <t xml:space="preserve">Don't need 50 workers a day; just 3–4 loaders plus cleaning staff</t>
   </si>
   <si>
-    <t xml:space="preserve">Farm workers removed from the packhouse. Loading, unloading &amp; cleaning = 3–4 loaders + 2 cleaners (₹0.12/kg).</t>
+    <t xml:space="preserve">Farm workers removed from the packhouse. Loading, unloading &amp; cleaning = 3–4 loaders + 2 cleaners (₹0.12/kg). Packhouse crew set to 20–30 workers (25 used).</t>
   </si>
   <si>
     <t xml:space="preserve">Procurement has no depreciation; premium costs ₹11 to grow, farmers charge ≤ ₹14; use ₹13.5; own farm earns ~₹3</t>
@@ -1163,7 +1181,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H84"/>
+  <dimension ref="A1:H86"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
@@ -1434,607 +1452,598 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="14" t="n">
-        <f aca="false">B21/(1-B12)-B21/(1-B11)</f>
-        <v>3.08771929824561</v>
-      </c>
-      <c r="C15" s="14" t="n">
-        <f aca="false">C21/(1-C12)-C21/(1-C11)</f>
-        <v>8.28947368421053</v>
-      </c>
-      <c r="D15" s="14" t="n">
-        <f aca="false">D21/(1-D12)-D21/(1-D11)</f>
-        <v>8.59649122807018</v>
+      <c r="B15" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>30</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F15" s="8"/>
       <c r="G15" s="8"/>
       <c r="H15" s="9" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B16" s="14" t="n">
-        <f aca="false">B21-B14</f>
-        <v>1</v>
-      </c>
-      <c r="C16" s="14" t="n">
-        <f aca="false">C21-C14</f>
-        <v>2.5</v>
-      </c>
-      <c r="D16" s="14" t="n">
-        <f aca="false">D21-D14</f>
-        <v>2</v>
+        <v>37</v>
+      </c>
+      <c r="B16" s="13" t="n">
+        <v>512.5</v>
+      </c>
+      <c r="C16" s="13" t="n">
+        <v>512.5</v>
+      </c>
+      <c r="D16" s="13" t="n">
+        <v>512.5</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="F16" s="8"/>
       <c r="G16" s="8"/>
       <c r="H16" s="9" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="B17" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="C17" s="16"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="16"/>
-      <c r="G17" s="16"/>
-      <c r="H17" s="16"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+    </row>
+    <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B19" s="4"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-    </row>
-    <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5" t="s">
+      <c r="B17" s="14" t="n">
+        <f aca="false">B23/(1-B12)-B23/(1-B11)</f>
+        <v>3.08771929824561</v>
+      </c>
+      <c r="C17" s="14" t="n">
+        <f aca="false">C23/(1-C12)-C23/(1-C11)</f>
+        <v>8.28947368421053</v>
+      </c>
+      <c r="D17" s="14" t="n">
+        <f aca="false">D23/(1-D12)-D23/(1-D11)</f>
+        <v>8.59649122807018</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="B20" s="5" t="s">
+    </row>
+    <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B18" s="14" t="n">
+        <f aca="false">B23-B14</f>
+        <v>1</v>
+      </c>
+      <c r="C18" s="14" t="n">
+        <f aca="false">C23-C14</f>
+        <v>2.5</v>
+      </c>
+      <c r="D18" s="14" t="n">
+        <f aca="false">D23-D14</f>
+        <v>2</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="B19" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="C19" s="16"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="16"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="16"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B21" s="4"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
+    </row>
+    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="C22" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D20" s="5" t="s">
+      <c r="D22" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E20" s="5" t="s">
+      <c r="E22" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F20" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="G20" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="H20" s="5" t="s">
+      <c r="F22" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="G22" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="H22" s="5" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B21" s="13" t="n">
-        <v>11</v>
-      </c>
-      <c r="C21" s="13" t="n">
-        <v>13.5</v>
-      </c>
-      <c r="D21" s="13" t="n">
-        <v>14</v>
-      </c>
-      <c r="E21" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="F21" s="14" t="n">
-        <f aca="false">C21</f>
-        <v>13.5</v>
-      </c>
-      <c r="G21" s="17" t="n">
-        <f aca="false">F21*$C$7*1000</f>
-        <v>162000</v>
-      </c>
-      <c r="H21" s="9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B22" s="14" t="n">
-        <f aca="false">B21*B11/(1-B11)</f>
-        <v>0.578947368421053</v>
-      </c>
-      <c r="C22" s="14" t="n">
-        <f aca="false">C21*C11/(1-C11)</f>
-        <v>0.710526315789474</v>
-      </c>
-      <c r="D22" s="14" t="n">
-        <f aca="false">D21*D11/(1-D11)</f>
-        <v>0.736842105263158</v>
-      </c>
-      <c r="E22" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="F22" s="14" t="n">
-        <f aca="false">C22</f>
-        <v>0.710526315789474</v>
-      </c>
-      <c r="G22" s="17" t="n">
-        <f aca="false">F22*$C$7*1000</f>
-        <v>8526.31578947369</v>
-      </c>
-      <c r="H22" s="9" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B23" s="13" t="n">
-        <v>0.8</v>
+        <v>11</v>
       </c>
       <c r="C23" s="13" t="n">
-        <v>1</v>
+        <v>13.5</v>
       </c>
       <c r="D23" s="13" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="E23" s="8" t="s">
         <v>32</v>
       </c>
       <c r="F23" s="14" t="n">
         <f aca="false">C23</f>
-        <v>1</v>
+        <v>13.5</v>
       </c>
       <c r="G23" s="17" t="n">
         <f aca="false">F23*$C$7*1000</f>
-        <v>12000</v>
+        <v>162000</v>
       </c>
       <c r="H23" s="9" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B24" s="13" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="C24" s="13" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D24" s="13" t="n">
-        <v>0.75</v>
+        <v>52</v>
+      </c>
+      <c r="B24" s="14" t="n">
+        <f aca="false">B23*B11/(1-B11)</f>
+        <v>0.578947368421053</v>
+      </c>
+      <c r="C24" s="14" t="n">
+        <f aca="false">C23*C11/(1-C11)</f>
+        <v>0.710526315789474</v>
+      </c>
+      <c r="D24" s="14" t="n">
+        <f aca="false">D23*D11/(1-D11)</f>
+        <v>0.736842105263158</v>
       </c>
       <c r="E24" s="8" t="s">
         <v>32</v>
       </c>
       <c r="F24" s="14" t="n">
         <f aca="false">C24</f>
-        <v>0.5</v>
+        <v>0.710526315789474</v>
       </c>
       <c r="G24" s="17" t="n">
         <f aca="false">F24*$C$7*1000</f>
-        <v>6000</v>
+        <v>8526.31578947369</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B25" s="13" t="n">
-        <v>0.45</v>
+        <v>0.8</v>
       </c>
       <c r="C25" s="13" t="n">
-        <v>0.55</v>
+        <v>1</v>
       </c>
       <c r="D25" s="13" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="E25" s="8" t="s">
         <v>32</v>
       </c>
       <c r="F25" s="14" t="n">
         <f aca="false">C25</f>
-        <v>0.55</v>
+        <v>1</v>
       </c>
       <c r="G25" s="17" t="n">
         <f aca="false">F25*$C$7*1000</f>
-        <v>6600</v>
+        <v>12000</v>
       </c>
       <c r="H25" s="9" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B26" s="13" t="n">
         <v>0.3</v>
       </c>
       <c r="C26" s="13" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="D26" s="13" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="E26" s="8" t="s">
         <v>32</v>
       </c>
       <c r="F26" s="14" t="n">
         <f aca="false">C26</f>
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="G26" s="17" t="n">
         <f aca="false">F26*$C$7*1000</f>
-        <v>4800</v>
+        <v>6000</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B27" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="C27" s="13" t="n">
-        <v>5.15</v>
-      </c>
-      <c r="D27" s="13" t="n">
-        <v>7.5</v>
+        <v>58</v>
+      </c>
+      <c r="B27" s="14" t="n">
+        <f aca="false">B15*B16/(B8*1000)</f>
+        <v>0.284722222222222</v>
+      </c>
+      <c r="C27" s="14" t="n">
+        <f aca="false">C15*C16/(C8*1000)</f>
+        <v>0.355902777777778</v>
+      </c>
+      <c r="D27" s="14" t="n">
+        <f aca="false">D15*D16/(D8*1000)</f>
+        <v>0.427083333333333</v>
       </c>
       <c r="E27" s="8" t="s">
         <v>32</v>
       </c>
       <c r="F27" s="14" t="n">
         <f aca="false">C27</f>
-        <v>5.15</v>
+        <v>0.355902777777778</v>
       </c>
       <c r="G27" s="17" t="n">
         <f aca="false">F27*$C$7*1000</f>
-        <v>61800</v>
+        <v>4270.83333333333</v>
       </c>
       <c r="H27" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B28" s="13" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="C28" s="13" t="n">
-        <v>0.26</v>
+        <v>0.4</v>
       </c>
       <c r="D28" s="13" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="E28" s="8" t="s">
         <v>32</v>
       </c>
       <c r="F28" s="14" t="n">
         <f aca="false">C28</f>
-        <v>0.26</v>
+        <v>0.4</v>
       </c>
       <c r="G28" s="17" t="n">
         <f aca="false">F28*$C$7*1000</f>
-        <v>3120</v>
+        <v>4800</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B29" s="13" t="n">
-        <v>0.08</v>
+        <v>1</v>
       </c>
       <c r="C29" s="13" t="n">
-        <v>0.12</v>
+        <v>5.15</v>
       </c>
       <c r="D29" s="13" t="n">
-        <v>0.15</v>
+        <v>7.5</v>
       </c>
       <c r="E29" s="8" t="s">
         <v>32</v>
       </c>
       <c r="F29" s="14" t="n">
         <f aca="false">C29</f>
-        <v>0.12</v>
+        <v>5.15</v>
       </c>
       <c r="G29" s="17" t="n">
         <f aca="false">F29*$C$7*1000</f>
-        <v>1440</v>
+        <v>61800</v>
       </c>
       <c r="H29" s="9" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B30" s="13" t="n">
-        <v>1.33</v>
+        <v>0.2</v>
       </c>
       <c r="C30" s="13" t="n">
-        <v>2.92</v>
+        <v>0.26</v>
       </c>
       <c r="D30" s="13" t="n">
-        <v>6.67</v>
+        <v>0.4</v>
       </c>
       <c r="E30" s="8" t="s">
         <v>32</v>
       </c>
       <c r="F30" s="14" t="n">
         <f aca="false">C30</f>
-        <v>2.92</v>
+        <v>0.26</v>
       </c>
       <c r="G30" s="17" t="n">
         <f aca="false">F30*$C$7*1000</f>
-        <v>35040</v>
+        <v>3120</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="B31" s="18" t="n">
-        <f aca="false">SUM(B21:B30)</f>
-        <v>16.0389473684211</v>
-      </c>
-      <c r="C31" s="18" t="n">
-        <f aca="false">SUM(C21:C30)</f>
-        <v>25.1105263157895</v>
-      </c>
-      <c r="D31" s="18" t="n">
-        <f aca="false">SUM(D21:D30)</f>
-        <v>32.4568421052632</v>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="B31" s="13" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="C31" s="13" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="D31" s="13" t="n">
+        <v>0.15</v>
       </c>
       <c r="E31" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F31" s="18" t="n">
+      <c r="F31" s="14" t="n">
         <f aca="false">C31</f>
-        <v>25.1105263157895</v>
-      </c>
-      <c r="G31" s="19" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G31" s="17" t="n">
         <f aca="false">F31*$C$7*1000</f>
-        <v>301326.315789474</v>
-      </c>
-      <c r="H31" s="8"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1440</v>
+      </c>
+      <c r="H31" s="9" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="B32" s="11" t="n">
+        <v>68</v>
+      </c>
+      <c r="B32" s="13" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="C32" s="13" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="D32" s="13" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="E32" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F32" s="14" t="n">
+        <f aca="false">C32</f>
+        <v>2.92</v>
+      </c>
+      <c r="G32" s="17" t="n">
+        <f aca="false">F32*$C$7*1000</f>
+        <v>35040</v>
+      </c>
+      <c r="H32" s="9" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="B33" s="18" t="n">
+        <f aca="false">SUM(B23:B32)</f>
+        <v>15.8736695906433</v>
+      </c>
+      <c r="C33" s="18" t="n">
+        <f aca="false">SUM(C23:C32)</f>
+        <v>24.9164290935673</v>
+      </c>
+      <c r="D33" s="18" t="n">
+        <f aca="false">SUM(D23:D32)</f>
+        <v>32.1339254385965</v>
+      </c>
+      <c r="E33" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F33" s="18" t="n">
+        <f aca="false">C33</f>
+        <v>24.9164290935673</v>
+      </c>
+      <c r="G33" s="19" t="n">
+        <f aca="false">F33*$C$7*1000</f>
+        <v>298997.149122807</v>
+      </c>
+      <c r="H33" s="8"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B34" s="11" t="n">
         <v>0.02</v>
       </c>
-      <c r="C32" s="11" t="n">
+      <c r="C34" s="11" t="n">
         <v>0.04</v>
       </c>
-      <c r="D32" s="11" t="n">
+      <c r="D34" s="11" t="n">
         <v>0.06</v>
       </c>
-      <c r="E32" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="F32" s="8"/>
-      <c r="G32" s="8"/>
-      <c r="H32" s="9" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B34" s="4"/>
-      <c r="C34" s="4"/>
-      <c r="D34" s="4"/>
-      <c r="E34" s="4"/>
-      <c r="F34" s="4"/>
-      <c r="G34" s="4"/>
-      <c r="H34" s="4"/>
-    </row>
-    <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="B35" s="5" t="s">
+      <c r="E34" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="F34" s="8"/>
+      <c r="G34" s="8"/>
+      <c r="H34" s="9" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B36" s="4"/>
+      <c r="C36" s="4"/>
+      <c r="D36" s="4"/>
+      <c r="E36" s="4"/>
+      <c r="F36" s="4"/>
+      <c r="G36" s="4"/>
+      <c r="H36" s="4"/>
+    </row>
+    <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B37" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C35" s="5" t="s">
+      <c r="C37" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D35" s="5" t="s">
+      <c r="D37" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E35" s="5" t="s">
+      <c r="E37" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F35" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="G35" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="H35" s="5" t="s">
+      <c r="F37" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="G37" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="H37" s="5" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="B36" s="20" t="n">
-        <v>18</v>
-      </c>
-      <c r="C36" s="20" t="n">
-        <v>24</v>
-      </c>
-      <c r="D36" s="20" t="n">
-        <v>30</v>
-      </c>
-      <c r="E36" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="F36" s="14" t="n">
-        <f aca="false">C36*100000/($C$10*1000)</f>
-        <v>0.222222222222222</v>
-      </c>
-      <c r="G36" s="17" t="n">
-        <f aca="false">F36*$C$7*1000</f>
-        <v>2666.66666666667</v>
-      </c>
-      <c r="H36" s="9" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="B37" s="20" t="n">
-        <v>8</v>
-      </c>
-      <c r="C37" s="20" t="n">
-        <v>12</v>
-      </c>
-      <c r="D37" s="20" t="n">
-        <v>15</v>
-      </c>
-      <c r="E37" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="F37" s="14" t="n">
-        <f aca="false">C37*100000/($C$10*1000)</f>
-        <v>0.111111111111111</v>
-      </c>
-      <c r="G37" s="17" t="n">
-        <f aca="false">F37*$C$7*1000</f>
-        <v>1333.33333333333</v>
-      </c>
-      <c r="H37" s="9" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B38" s="20" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="C38" s="20" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="D38" s="20" t="n">
-        <v>3.5</v>
+        <v>30</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="F38" s="14" t="n">
         <f aca="false">C38*100000/($C$10*1000)</f>
-        <v>0.0185185185185185</v>
+        <v>0.222222222222222</v>
       </c>
       <c r="G38" s="17" t="n">
         <f aca="false">F38*$C$7*1000</f>
-        <v>222.222222222222</v>
+        <v>2666.66666666667</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B39" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="C39" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="D39" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="E39" s="8" t="s">
         <v>76</v>
-      </c>
-      <c r="B39" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="C39" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="D39" s="20" t="n">
-        <v>8</v>
-      </c>
-      <c r="E39" s="8" t="s">
-        <v>70</v>
       </c>
       <c r="F39" s="14" t="n">
         <f aca="false">C39*100000/($C$10*1000)</f>
-        <v>0.0555555555555556</v>
+        <v>0.111111111111111</v>
       </c>
       <c r="G39" s="17" t="n">
         <f aca="false">F39*$C$7*1000</f>
-        <v>666.666666666667</v>
+        <v>1333.33333333333</v>
       </c>
       <c r="H39" s="9" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B40" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C40" s="20" t="n">
         <v>2</v>
       </c>
       <c r="D40" s="20" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="F40" s="14" t="n">
         <f aca="false">C40*100000/($C$10*1000)</f>
@@ -2045,349 +2054,363 @@
         <v>222.222222222222</v>
       </c>
       <c r="H40" s="9" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="B41" s="12" t="n">
-        <f aca="false">B61/B71</f>
-        <v>13.3</v>
-      </c>
-      <c r="C41" s="12" t="n">
-        <f aca="false">C61/C71</f>
-        <v>21.1365</v>
-      </c>
-      <c r="D41" s="12" t="n">
-        <f aca="false">D61/D71</f>
-        <v>33.99375</v>
+        <v>82</v>
+      </c>
+      <c r="B41" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="C41" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="D41" s="20" t="n">
+        <v>8</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="F41" s="14" t="n">
         <f aca="false">C41*100000/($C$10*1000)</f>
-        <v>0.195708333333333</v>
+        <v>0.0555555555555556</v>
       </c>
       <c r="G41" s="17" t="n">
         <f aca="false">F41*$C$7*1000</f>
-        <v>2348.5</v>
+        <v>666.666666666667</v>
       </c>
       <c r="H41" s="9" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="B42" s="12" t="n">
-        <f aca="false">B63*B68*B69+B66*B70</f>
-        <v>9.77481473684211</v>
-      </c>
-      <c r="C42" s="12" t="n">
-        <f aca="false">C63*C68*C69+C66*C70</f>
-        <v>26.787309868421</v>
-      </c>
-      <c r="D42" s="12" t="n">
-        <f aca="false">D63*D68*D69+D66*D70</f>
-        <v>60.668237368421</v>
+        <v>84</v>
+      </c>
+      <c r="B42" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D42" s="20" t="n">
+        <v>3</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="F42" s="14" t="n">
         <f aca="false">C42*100000/($C$10*1000)</f>
-        <v>0.248030646929825</v>
+        <v>0.0185185185185185</v>
       </c>
       <c r="G42" s="17" t="n">
         <f aca="false">F42*$C$7*1000</f>
+        <v>222.222222222222</v>
+      </c>
+      <c r="H42" s="9" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B43" s="12" t="n">
+        <f aca="false">B63/B73</f>
+        <v>13.3</v>
+      </c>
+      <c r="C43" s="12" t="n">
+        <f aca="false">C63/C73</f>
+        <v>21.1365</v>
+      </c>
+      <c r="D43" s="12" t="n">
+        <f aca="false">D63/D73</f>
+        <v>33.99375</v>
+      </c>
+      <c r="E43" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="F43" s="14" t="n">
+        <f aca="false">C43*100000/($C$10*1000)</f>
+        <v>0.195708333333333</v>
+      </c>
+      <c r="G43" s="17" t="n">
+        <f aca="false">F43*$C$7*1000</f>
+        <v>2348.5</v>
+      </c>
+      <c r="H43" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B44" s="12" t="n">
+        <f aca="false">B65*B70*B71+B68*B72</f>
+        <v>9.77481473684211</v>
+      </c>
+      <c r="C44" s="12" t="n">
+        <f aca="false">C65*C70*C71+C68*C72</f>
+        <v>26.787309868421</v>
+      </c>
+      <c r="D44" s="12" t="n">
+        <f aca="false">D65*D70*D71+D68*D72</f>
+        <v>60.668237368421</v>
+      </c>
+      <c r="E44" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="F44" s="14" t="n">
+        <f aca="false">C44*100000/($C$10*1000)</f>
+        <v>0.248030646929825</v>
+      </c>
+      <c r="G44" s="17" t="n">
+        <f aca="false">F44*$C$7*1000</f>
         <v>2976.36776315789</v>
       </c>
-      <c r="H42" s="9" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="15" t="s">
-        <v>84</v>
-      </c>
-      <c r="B43" s="21" t="n">
-        <f aca="false">SUM(B36:B42)</f>
+      <c r="H44" s="9" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="B45" s="21" t="n">
+        <f aca="false">SUM(B38:B44)</f>
         <v>54.0748147368421</v>
       </c>
-      <c r="C43" s="21" t="n">
-        <f aca="false">SUM(C36:C42)</f>
+      <c r="C45" s="21" t="n">
+        <f aca="false">SUM(C38:C44)</f>
         <v>93.9238098684211</v>
       </c>
-      <c r="D43" s="21" t="n">
-        <f aca="false">SUM(D36:D42)</f>
+      <c r="D45" s="21" t="n">
+        <f aca="false">SUM(D38:D44)</f>
         <v>154.161987368421</v>
       </c>
-      <c r="E43" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="F43" s="18" t="n">
-        <f aca="false">C43*100000/($C$10*1000)</f>
+      <c r="E45" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="F45" s="18" t="n">
+        <f aca="false">C45*100000/($C$10*1000)</f>
         <v>0.869664906189084</v>
       </c>
-      <c r="G43" s="19" t="n">
-        <f aca="false">F43*$C$7*1000</f>
+      <c r="G45" s="19" t="n">
+        <f aca="false">F45*$C$7*1000</f>
         <v>10435.978874269</v>
       </c>
-      <c r="H43" s="9" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="B44" s="22" t="n">
-        <f aca="false">B43*100000/(B10*1000)</f>
+      <c r="H45" s="9" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="B46" s="22" t="n">
+        <f aca="false">B45*100000/(B10*1000)</f>
         <v>0.55632525449426</v>
       </c>
-      <c r="C44" s="22" t="n">
-        <f aca="false">C43*100000/(C10*1000)</f>
+      <c r="C46" s="22" t="n">
+        <f aca="false">C45*100000/(C10*1000)</f>
         <v>0.869664906189084</v>
       </c>
-      <c r="D44" s="22" t="n">
-        <f aca="false">D43*100000/(D10*1000)</f>
+      <c r="D46" s="22" t="n">
+        <f aca="false">D45*100000/(D10*1000)</f>
         <v>1.29765982633351</v>
       </c>
-      <c r="E44" s="8" t="s">
+      <c r="E46" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F44" s="8"/>
-      <c r="G44" s="8"/>
-      <c r="H44" s="9" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="B46" s="4"/>
-      <c r="C46" s="4"/>
-      <c r="D46" s="4"/>
-      <c r="E46" s="4"/>
-      <c r="F46" s="4"/>
-      <c r="G46" s="4"/>
-      <c r="H46" s="4"/>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="15" t="s">
-        <v>89</v>
-      </c>
-      <c r="B47" s="18" t="n">
-        <f aca="false">B31+B44</f>
-        <v>16.5952726229153</v>
-      </c>
-      <c r="C47" s="18" t="n">
-        <f aca="false">C31+C44</f>
-        <v>25.9801912219786</v>
-      </c>
-      <c r="D47" s="18" t="n">
-        <f aca="false">D31+D44</f>
-        <v>33.7545019315967</v>
-      </c>
-      <c r="E47" s="8" t="s">
+      <c r="F46" s="8"/>
+      <c r="G46" s="8"/>
+      <c r="H46" s="9" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B48" s="4"/>
+      <c r="C48" s="4"/>
+      <c r="D48" s="4"/>
+      <c r="E48" s="4"/>
+      <c r="F48" s="4"/>
+      <c r="G48" s="4"/>
+      <c r="H48" s="4"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="B49" s="18" t="n">
+        <f aca="false">B33+B46</f>
+        <v>16.4299948451375</v>
+      </c>
+      <c r="C49" s="18" t="n">
+        <f aca="false">C33+C46</f>
+        <v>25.7860939997563</v>
+      </c>
+      <c r="D49" s="18" t="n">
+        <f aca="false">D33+D46</f>
+        <v>33.43158526493</v>
+      </c>
+      <c r="E49" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F47" s="18" t="n">
-        <f aca="false">C47</f>
-        <v>25.9801912219786</v>
-      </c>
-      <c r="G47" s="19" t="n">
-        <f aca="false">F47*$C$7*1000</f>
-        <v>311762.294663743</v>
-      </c>
-      <c r="H47" s="9" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="B49" s="4"/>
-      <c r="C49" s="4"/>
-      <c r="D49" s="4"/>
-      <c r="E49" s="4"/>
-      <c r="F49" s="4"/>
-      <c r="G49" s="4"/>
-      <c r="H49" s="4"/>
-    </row>
-    <row r="50" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="B50" s="5" t="s">
+      <c r="F49" s="18" t="n">
+        <f aca="false">C49</f>
+        <v>25.7860939997563</v>
+      </c>
+      <c r="G49" s="19" t="n">
+        <f aca="false">F49*$C$7*1000</f>
+        <v>309433.127997076</v>
+      </c>
+      <c r="H49" s="9" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B51" s="4"/>
+      <c r="C51" s="4"/>
+      <c r="D51" s="4"/>
+      <c r="E51" s="4"/>
+      <c r="F51" s="4"/>
+      <c r="G51" s="4"/>
+      <c r="H51" s="4"/>
+    </row>
+    <row r="52" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B52" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C50" s="5" t="s">
+      <c r="C52" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D50" s="5" t="s">
+      <c r="D52" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E50" s="5" t="s">
+      <c r="E52" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F50" s="5"/>
-      <c r="G50" s="5"/>
-      <c r="H50" s="5" t="s">
+      <c r="F52" s="5"/>
+      <c r="G52" s="5"/>
+      <c r="H52" s="5" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="B51" s="20" t="n">
-        <v>60</v>
-      </c>
-      <c r="C51" s="20" t="n">
-        <v>75</v>
-      </c>
-      <c r="D51" s="20" t="n">
-        <v>90</v>
-      </c>
-      <c r="E51" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="F51" s="8"/>
-      <c r="G51" s="8"/>
-      <c r="H51" s="9" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="B52" s="20" t="n">
-        <v>50</v>
-      </c>
-      <c r="C52" s="20" t="n">
-        <v>60</v>
-      </c>
-      <c r="D52" s="20" t="n">
-        <v>90</v>
-      </c>
-      <c r="E52" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="F52" s="8"/>
-      <c r="G52" s="8"/>
-      <c r="H52" s="9" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B53" s="20" t="n">
-        <v>6</v>
+        <v>60</v>
       </c>
       <c r="C53" s="20" t="n">
-        <v>8.8</v>
+        <v>75</v>
       </c>
       <c r="D53" s="20" t="n">
-        <v>12</v>
+        <v>90</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F53" s="8"/>
       <c r="G53" s="8"/>
       <c r="H53" s="9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B54" s="20" t="n">
+        <v>50</v>
+      </c>
+      <c r="C54" s="20" t="n">
+        <v>60</v>
+      </c>
+      <c r="D54" s="20" t="n">
+        <v>90</v>
+      </c>
+      <c r="E54" s="8" t="s">
         <v>100</v>
-      </c>
-      <c r="B54" s="20" t="n">
-        <v>8</v>
-      </c>
-      <c r="C54" s="20" t="n">
-        <v>12</v>
-      </c>
-      <c r="D54" s="20" t="n">
-        <v>14</v>
-      </c>
-      <c r="E54" s="8" t="s">
-        <v>94</v>
       </c>
       <c r="F54" s="8"/>
       <c r="G54" s="8"/>
       <c r="H54" s="9" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="6" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B55" s="20" t="n">
         <v>6</v>
       </c>
       <c r="C55" s="20" t="n">
-        <v>10</v>
+        <v>8.8</v>
       </c>
       <c r="D55" s="20" t="n">
         <v>12</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F55" s="8"/>
       <c r="G55" s="8"/>
-      <c r="H55" s="9"/>
+      <c r="H55" s="9" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="6" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B56" s="20" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C56" s="20" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D56" s="20" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="E56" s="8" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F56" s="8"/>
       <c r="G56" s="8"/>
       <c r="H56" s="9" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="6" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B57" s="20" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C57" s="20" t="n">
-        <v>10.5</v>
+        <v>10</v>
       </c>
       <c r="D57" s="20" t="n">
         <v>12</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F57" s="8"/>
       <c r="G57" s="8"/>
@@ -2395,39 +2418,41 @@
     </row>
     <row r="58" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="6" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B58" s="20" t="n">
         <v>5</v>
       </c>
       <c r="C58" s="20" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D58" s="20" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E58" s="8" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F58" s="8"/>
       <c r="G58" s="8"/>
-      <c r="H58" s="9"/>
+      <c r="H58" s="9" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="6" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B59" s="20" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C59" s="20" t="n">
-        <v>10</v>
+        <v>10.5</v>
       </c>
       <c r="D59" s="20" t="n">
         <v>12</v>
       </c>
       <c r="E59" s="8" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F59" s="8"/>
       <c r="G59" s="8"/>
@@ -2435,47 +2460,39 @@
     </row>
     <row r="60" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="B60" s="12" t="n">
-        <f aca="false">SUM(B51:B59)*5%</f>
-        <v>7.6</v>
-      </c>
-      <c r="C60" s="12" t="n">
-        <f aca="false">SUM(C51:C59)*5%</f>
-        <v>10.065</v>
-      </c>
-      <c r="D60" s="12" t="n">
-        <f aca="false">SUM(D51:D59)*5%</f>
-        <v>12.95</v>
+        <v>112</v>
+      </c>
+      <c r="B60" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="C60" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="D60" s="20" t="n">
+        <v>9</v>
       </c>
       <c r="E60" s="8" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F60" s="8"/>
       <c r="G60" s="8"/>
-      <c r="H60" s="9" t="s">
-        <v>109</v>
-      </c>
+      <c r="H60" s="9"/>
     </row>
     <row r="61" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="B61" s="23" t="n">
-        <f aca="false">SUM(B51:B60)</f>
-        <v>159.6</v>
-      </c>
-      <c r="C61" s="23" t="n">
-        <f aca="false">SUM(C51:C60)</f>
-        <v>211.365</v>
-      </c>
-      <c r="D61" s="23" t="n">
-        <f aca="false">SUM(D51:D60)</f>
-        <v>271.95</v>
+        <v>113</v>
+      </c>
+      <c r="B61" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="C61" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="D61" s="20" t="n">
+        <v>12</v>
       </c>
       <c r="E61" s="8" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F61" s="8"/>
       <c r="G61" s="8"/>
@@ -2483,47 +2500,47 @@
     </row>
     <row r="62" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="6" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B62" s="12" t="n">
-        <f aca="false">-35%*(MIN(B51,50)+MIN(B52,50)+MIN(B53,3.2))</f>
-        <v>-36.12</v>
+        <f aca="false">SUM(B53:B61)*5%</f>
+        <v>7.6</v>
       </c>
       <c r="C62" s="12" t="n">
-        <f aca="false">-35%*(MIN(C51,50)+MIN(C52,50)+MIN(C53,3.2))</f>
-        <v>-36.12</v>
+        <f aca="false">SUM(C53:C61)*5%</f>
+        <v>10.065</v>
       </c>
       <c r="D62" s="12" t="n">
-        <f aca="false">-35%*(MIN(D51,50)+MIN(D52,50)+MIN(D53,3.2))</f>
-        <v>-36.12</v>
+        <f aca="false">SUM(D53:D61)*5%</f>
+        <v>12.95</v>
       </c>
       <c r="E62" s="8" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F62" s="8"/>
       <c r="G62" s="8"/>
       <c r="H62" s="9" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="B63" s="12" t="n">
-        <f aca="false">B61+B62</f>
-        <v>123.48</v>
-      </c>
-      <c r="C63" s="12" t="n">
-        <f aca="false">C61+C62</f>
-        <v>175.245</v>
-      </c>
-      <c r="D63" s="12" t="n">
-        <f aca="false">D61+D62</f>
-        <v>235.83</v>
+        <v>116</v>
+      </c>
+      <c r="B63" s="23" t="n">
+        <f aca="false">SUM(B53:B62)</f>
+        <v>159.6</v>
+      </c>
+      <c r="C63" s="23" t="n">
+        <f aca="false">SUM(C53:C62)</f>
+        <v>211.365</v>
+      </c>
+      <c r="D63" s="23" t="n">
+        <f aca="false">SUM(D53:D62)</f>
+        <v>271.95</v>
       </c>
       <c r="E63" s="8" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F63" s="8"/>
       <c r="G63" s="8"/>
@@ -2531,135 +2548,139 @@
     </row>
     <row r="64" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="B64" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="C64" s="7" t="n">
-        <v>21</v>
-      </c>
-      <c r="D64" s="7" t="n">
-        <v>45</v>
+        <v>117</v>
+      </c>
+      <c r="B64" s="12" t="n">
+        <f aca="false">-35%*(MIN(B53,50)+MIN(B54,50)+MIN(B55,3.2))</f>
+        <v>-36.12</v>
+      </c>
+      <c r="C64" s="12" t="n">
+        <f aca="false">-35%*(MIN(C53,50)+MIN(C54,50)+MIN(C55,3.2))</f>
+        <v>-36.12</v>
+      </c>
+      <c r="D64" s="12" t="n">
+        <f aca="false">-35%*(MIN(D53,50)+MIN(D54,50)+MIN(D55,3.2))</f>
+        <v>-36.12</v>
       </c>
       <c r="E64" s="8" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="F64" s="8"/>
       <c r="G64" s="8"/>
       <c r="H64" s="9" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="B65" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="C65" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="D65" s="7" t="n">
-        <v>7</v>
+        <v>119</v>
+      </c>
+      <c r="B65" s="12" t="n">
+        <f aca="false">B63+B64</f>
+        <v>123.48</v>
+      </c>
+      <c r="C65" s="12" t="n">
+        <f aca="false">C63+C64</f>
+        <v>175.245</v>
+      </c>
+      <c r="D65" s="12" t="n">
+        <f aca="false">D63+D64</f>
+        <v>235.83</v>
       </c>
       <c r="E65" s="8" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="F65" s="8"/>
       <c r="G65" s="8"/>
-      <c r="H65" s="9" t="s">
-        <v>118</v>
-      </c>
+      <c r="H65" s="9"/>
     </row>
     <row r="66" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="B66" s="12" t="n">
-        <f aca="false">(B64*B8*1000*$C$76-B65*B13*1000*B21)/100000</f>
-        <v>41.3810526315789</v>
-      </c>
-      <c r="C66" s="12" t="n">
-        <f aca="false">(C64*C8*1000*$C$76-C65*C13*1000*C21)/100000</f>
-        <v>175.869473684211</v>
-      </c>
-      <c r="D66" s="12" t="n">
-        <f aca="false">(D64*D8*1000*$C$76-D65*D13*1000*D21)/100000</f>
-        <v>416.463157894737</v>
+        <v>120</v>
+      </c>
+      <c r="B66" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="C66" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="D66" s="7" t="n">
+        <v>45</v>
       </c>
       <c r="E66" s="8" t="s">
-        <v>94</v>
+        <v>121</v>
       </c>
       <c r="F66" s="8"/>
       <c r="G66" s="8"/>
       <c r="H66" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="B67" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="C67" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="D67" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="E67" s="8" t="s">
         <v>121</v>
-      </c>
-      <c r="B67" s="24" t="n">
-        <f aca="false">B63+B66</f>
-        <v>164.861052631579</v>
-      </c>
-      <c r="C67" s="24" t="n">
-        <f aca="false">C63+C66</f>
-        <v>351.114473684211</v>
-      </c>
-      <c r="D67" s="24" t="n">
-        <f aca="false">D63+D66</f>
-        <v>652.293157894737</v>
-      </c>
-      <c r="E67" s="8" t="s">
-        <v>94</v>
       </c>
       <c r="F67" s="8"/>
       <c r="G67" s="8"/>
       <c r="H67" s="9" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="B68" s="11" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="C68" s="11" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="D68" s="11" t="n">
-        <v>0.7</v>
+        <v>125</v>
+      </c>
+      <c r="B68" s="12" t="n">
+        <f aca="false">(B66*B8*1000*$C$78-B67*B13*1000*B23)/100000</f>
+        <v>41.3810526315789</v>
+      </c>
+      <c r="C68" s="12" t="n">
+        <f aca="false">(C66*C8*1000*$C$78-C67*C13*1000*C23)/100000</f>
+        <v>175.869473684211</v>
+      </c>
+      <c r="D68" s="12" t="n">
+        <f aca="false">(D66*D8*1000*$C$78-D67*D13*1000*D23)/100000</f>
+        <v>416.463157894737</v>
       </c>
       <c r="E68" s="8" t="s">
-        <v>124</v>
+        <v>100</v>
       </c>
       <c r="F68" s="8"/>
       <c r="G68" s="8"/>
       <c r="H68" s="9" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="B69" s="25" t="n">
-        <v>0.07</v>
-      </c>
-      <c r="C69" s="25" t="n">
-        <v>0.075</v>
-      </c>
-      <c r="D69" s="25" t="n">
-        <v>0.09</v>
+        <v>127</v>
+      </c>
+      <c r="B69" s="24" t="n">
+        <f aca="false">B65+B68</f>
+        <v>164.861052631579</v>
+      </c>
+      <c r="C69" s="24" t="n">
+        <f aca="false">C65+C68</f>
+        <v>351.114473684211</v>
+      </c>
+      <c r="D69" s="24" t="n">
+        <f aca="false">D65+D68</f>
+        <v>652.293157894737</v>
       </c>
       <c r="E69" s="8" t="s">
-        <v>127</v>
+        <v>100</v>
       </c>
       <c r="F69" s="8"/>
       <c r="G69" s="8"/>
@@ -2671,222 +2692,216 @@
       <c r="A70" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="B70" s="25" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="C70" s="25" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D70" s="25" t="n">
-        <v>0.11</v>
+      <c r="B70" s="11" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="C70" s="11" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D70" s="11" t="n">
+        <v>0.7</v>
       </c>
       <c r="E70" s="8" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="F70" s="8"/>
       <c r="G70" s="8"/>
       <c r="H70" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="B71" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="C71" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="D71" s="7" t="n">
-        <v>8</v>
+        <v>132</v>
+      </c>
+      <c r="B71" s="25" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="C71" s="25" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="D71" s="25" t="n">
+        <v>0.09</v>
       </c>
       <c r="E71" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F71" s="8"/>
       <c r="G71" s="8"/>
       <c r="H71" s="9" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="B72" s="25" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="C72" s="25" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D72" s="25" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="E72" s="8" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="B73" s="4"/>
-      <c r="C73" s="4"/>
-      <c r="D73" s="4"/>
-      <c r="E73" s="4"/>
-      <c r="F73" s="4"/>
-      <c r="G73" s="4"/>
-      <c r="H73" s="4"/>
-    </row>
-    <row r="74" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="B74" s="5" t="s">
+      <c r="F72" s="8"/>
+      <c r="G72" s="8"/>
+      <c r="H72" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="C74" s="5" t="s">
+    </row>
+    <row r="73" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A73" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="B73" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="C73" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D73" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="E73" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="F73" s="8"/>
+      <c r="G73" s="8"/>
+      <c r="H73" s="9" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B75" s="4"/>
+      <c r="C75" s="4"/>
+      <c r="D75" s="4"/>
+      <c r="E75" s="4"/>
+      <c r="F75" s="4"/>
+      <c r="G75" s="4"/>
+      <c r="H75" s="4"/>
+    </row>
+    <row r="76" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A76" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="B76" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="C76" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D74" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="E74" s="5" t="s">
+      <c r="D76" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="E76" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F74" s="5"/>
-      <c r="G74" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="H74" s="5" t="s">
+      <c r="F76" s="5"/>
+      <c r="G76" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="H76" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A75" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="B75" s="10" t="n">
+    <row r="77" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A77" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="B77" s="10" t="n">
         <f aca="false">B10</f>
         <v>9720</v>
       </c>
-      <c r="C75" s="10" t="n">
+      <c r="C77" s="10" t="n">
         <f aca="false">C10</f>
         <v>10800</v>
       </c>
-      <c r="D75" s="10" t="n">
+      <c r="D77" s="10" t="n">
         <f aca="false">D10</f>
         <v>11880</v>
       </c>
-      <c r="E75" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="F75" s="8"/>
-      <c r="G75" s="8"/>
-      <c r="H75" s="9" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="76" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A76" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="B76" s="13" t="n">
-        <v>24</v>
-      </c>
-      <c r="C76" s="13" t="n">
-        <v>28</v>
-      </c>
-      <c r="D76" s="13" t="n">
-        <v>32</v>
-      </c>
-      <c r="E76" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="F76" s="8"/>
-      <c r="G76" s="17" t="n">
-        <f aca="false">C76*$C$7*1000</f>
-        <v>336000</v>
-      </c>
-      <c r="H76" s="9" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="77" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A77" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="B77" s="12" t="n">
-        <f aca="false">$C$76*B10*1000/100000</f>
-        <v>2721.6</v>
-      </c>
-      <c r="C77" s="12" t="n">
-        <f aca="false">$C$76*C10*1000/100000</f>
-        <v>3024</v>
-      </c>
-      <c r="D77" s="12" t="n">
-        <f aca="false">$C$76*D10*1000/100000</f>
-        <v>3326.4</v>
-      </c>
       <c r="E77" s="8" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
       <c r="F77" s="8"/>
       <c r="G77" s="8"/>
       <c r="H77" s="9" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="B78" s="26" t="n">
-        <f aca="false">B47/(1-B32)</f>
-        <v>16.933951656036</v>
-      </c>
-      <c r="C78" s="26" t="n">
-        <f aca="false">C47/(1-C32)</f>
-        <v>27.062699189561</v>
-      </c>
-      <c r="D78" s="26" t="n">
-        <f aca="false">D47/(1-D32)</f>
-        <v>35.9090446080816</v>
+        <v>148</v>
+      </c>
+      <c r="B78" s="13" t="n">
+        <v>24</v>
+      </c>
+      <c r="C78" s="13" t="n">
+        <v>28</v>
+      </c>
+      <c r="D78" s="13" t="n">
+        <v>32</v>
       </c>
       <c r="E78" s="8" t="s">
         <v>32</v>
       </c>
       <c r="F78" s="8"/>
-      <c r="G78" s="27" t="n">
+      <c r="G78" s="17" t="n">
         <f aca="false">C78*$C$7*1000</f>
-        <v>324752.390274732</v>
+        <v>336000</v>
       </c>
       <c r="H78" s="9" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="15" t="s">
-        <v>148</v>
-      </c>
-      <c r="B79" s="11" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="C79" s="11" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D79" s="11" t="n">
-        <v>0.1</v>
+        <v>149</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="B79" s="12" t="n">
+        <f aca="false">$C$78*B10*1000/100000</f>
+        <v>2721.6</v>
+      </c>
+      <c r="C79" s="12" t="n">
+        <f aca="false">$C$78*C10*1000/100000</f>
+        <v>3024</v>
+      </c>
+      <c r="D79" s="12" t="n">
+        <f aca="false">$C$78*D10*1000/100000</f>
+        <v>3326.4</v>
       </c>
       <c r="E79" s="8" t="s">
-        <v>149</v>
+        <v>100</v>
       </c>
       <c r="F79" s="8"/>
       <c r="G79" s="8"/>
-      <c r="H79" s="8" t="s">
-        <v>150</v>
+      <c r="H79" s="9" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B80" s="26" t="n">
-        <f aca="false">B47/(1-B32-B79)</f>
-        <v>18.8582643442219</v>
+        <f aca="false">B49/(1-B34)</f>
+        <v>16.7653008623852</v>
       </c>
       <c r="C80" s="26" t="n">
-        <f aca="false">C47/(1-C32-C79)</f>
-        <v>30.2095246767193</v>
+        <f aca="false">C49/(1-C34)</f>
+        <v>26.8605145830795</v>
       </c>
       <c r="D80" s="26" t="n">
-        <f aca="false">D47/(1-D32-D79)</f>
-        <v>40.1839308709484</v>
+        <f aca="false">D49/(1-D34)</f>
+        <v>35.5655162392872</v>
       </c>
       <c r="E80" s="8" t="s">
         <v>32</v>
@@ -2894,110 +2909,160 @@
       <c r="F80" s="8"/>
       <c r="G80" s="27" t="n">
         <f aca="false">C80*$C$7*1000</f>
-        <v>362514.296120631</v>
+        <v>322326.174996954</v>
       </c>
       <c r="H80" s="9" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A81" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="B81" s="22" t="n">
-        <f aca="false">$C$76*(1-B32)-B47</f>
-        <v>10.8447273770847</v>
-      </c>
-      <c r="C81" s="22" t="n">
-        <f aca="false">$C$76*(1-C32)-C47</f>
-        <v>0.899808778021441</v>
-      </c>
-      <c r="D81" s="22" t="n">
-        <f aca="false">$C$76*(1-D32)-D47</f>
-        <v>-7.43450193159666</v>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="B81" s="11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C81" s="11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D81" s="11" t="n">
+        <v>0.1</v>
       </c>
       <c r="E81" s="8" t="s">
-        <v>32</v>
+        <v>155</v>
       </c>
       <c r="F81" s="8"/>
-      <c r="G81" s="28" t="n">
-        <f aca="false">C81*$C$7*1000</f>
-        <v>10797.7053362573</v>
-      </c>
-      <c r="H81" s="9" t="s">
-        <v>154</v>
+      <c r="G81" s="8"/>
+      <c r="H81" s="8" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="B82" s="29" t="n">
-        <f aca="false">B81*B10*1000/100000</f>
-        <v>1054.10750105263</v>
-      </c>
-      <c r="C82" s="29" t="n">
-        <f aca="false">C81*C10*1000/100000</f>
-        <v>97.1793480263157</v>
-      </c>
-      <c r="D82" s="29" t="n">
-        <f aca="false">D81*D10*1000/100000</f>
-        <v>-883.218829473684</v>
+        <v>157</v>
+      </c>
+      <c r="B82" s="26" t="n">
+        <f aca="false">B49/(1-B34-B81)</f>
+        <v>18.6704486876563</v>
+      </c>
+      <c r="C82" s="26" t="n">
+        <f aca="false">C49/(1-C34-C81)</f>
+        <v>29.9838302322748</v>
+      </c>
+      <c r="D82" s="26" t="n">
+        <f aca="false">D49/(1-D34-D81)</f>
+        <v>39.7995062677738</v>
       </c>
       <c r="E82" s="8" t="s">
-        <v>94</v>
+        <v>32</v>
       </c>
       <c r="F82" s="8"/>
-      <c r="G82" s="30"/>
+      <c r="G82" s="27" t="n">
+        <f aca="false">C82*$C$7*1000</f>
+        <v>359805.962787298</v>
+      </c>
       <c r="H82" s="9" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="B83" s="12" t="n">
-        <f aca="false">IF(B82+B41&lt;=0,"Not recovered",B67/(B82+B41))</f>
-        <v>0.154449966361488</v>
-      </c>
-      <c r="C83" s="12" t="n">
-        <f aca="false">IF(C82+C41&lt;=0,"Not recovered",C67/(C82+C41))</f>
-        <v>2.96760306874626</v>
-      </c>
-      <c r="D83" s="12" t="str">
-        <f aca="false">IF(D82+D41&lt;=0,"Not recovered",D67/(D82+D41))</f>
+        <v>159</v>
+      </c>
+      <c r="B83" s="22" t="n">
+        <f aca="false">$C$78*(1-B34)-B49</f>
+        <v>11.0100051548625</v>
+      </c>
+      <c r="C83" s="22" t="n">
+        <f aca="false">$C$78*(1-C34)-C49</f>
+        <v>1.09390600024366</v>
+      </c>
+      <c r="D83" s="22" t="n">
+        <f aca="false">$C$78*(1-D34)-D49</f>
+        <v>-7.11158526493</v>
+      </c>
+      <c r="E83" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F83" s="8"/>
+      <c r="G83" s="28" t="n">
+        <f aca="false">C83*$C$7*1000</f>
+        <v>13126.872002924</v>
+      </c>
+      <c r="H83" s="9" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A84" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="B84" s="29" t="n">
+        <f aca="false">B83*B10*1000/100000</f>
+        <v>1070.17250105263</v>
+      </c>
+      <c r="C84" s="29" t="n">
+        <f aca="false">C83*C10*1000/100000</f>
+        <v>118.141848026316</v>
+      </c>
+      <c r="D84" s="29" t="n">
+        <f aca="false">D83*D10*1000/100000</f>
+        <v>-844.856329473684</v>
+      </c>
+      <c r="E84" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="F84" s="8"/>
+      <c r="G84" s="30"/>
+      <c r="H84" s="9" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A85" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="B85" s="12" t="n">
+        <f aca="false">IF(B84+B43&lt;=0,"Not recovered",B69/(B84+B43))</f>
+        <v>0.152159886357439</v>
+      </c>
+      <c r="C85" s="12" t="n">
+        <f aca="false">IF(C84+C43&lt;=0,"Not recovered",C69/(C84+C43))</f>
+        <v>2.52095518549567</v>
+      </c>
+      <c r="D85" s="12" t="str">
+        <f aca="false">IF(D84+D43&lt;=0,"Not recovered",D69/(D84+D43))</f>
         <v>Not recovered</v>
       </c>
-      <c r="E83" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="F83" s="8"/>
-      <c r="G83" s="8"/>
-      <c r="H83" s="9" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="84" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A84" s="15" t="s">
-        <v>159</v>
-      </c>
-      <c r="B84" s="16" t="str">
-        <f aca="false">"We put in ₹"&amp;TEXT(C67,"#,##0")&amp;" L and sell "&amp;TEXT(C75,"#,##0")&amp;" t a year. Break-even is ₹"&amp;TEXT(C78,"0.00")&amp;"/kg and ₹"&amp;TEXT(C80,"0.00")&amp;"/kg earns a "&amp;TEXT(C79,"0%")&amp;" margin. At ₹"&amp;TEXT(C76,"0")&amp;"/kg we make ₹"&amp;TEXT(C82,"#,##0.0")&amp;" L a year. Every ₹1/kg higher price adds ₹"&amp;TEXT(C10*1000*(1-C32)/100000,"#,##0")&amp;" L a year."</f>
-        <v>We put in ₹351 L and sell 10,800 t a year. Break-even is ₹27.06/kg and ₹30.21/kg earns a 10% margin. At ₹28/kg we make ₹97.2 L a year. Every ₹1/kg higher price adds ₹104 L a year.</v>
-      </c>
-      <c r="C84" s="16"/>
-      <c r="D84" s="16"/>
-      <c r="E84" s="16"/>
-      <c r="F84" s="16"/>
-      <c r="G84" s="16"/>
-      <c r="H84" s="16"/>
+      <c r="E85" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="F85" s="8"/>
+      <c r="G85" s="8"/>
+      <c r="H85" s="9" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A86" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="B86" s="16" t="str">
+        <f aca="false">"We put in ₹"&amp;TEXT(C69,"#,##0")&amp;" L and sell "&amp;TEXT(C77,"#,##0")&amp;" t a year. Break-even is ₹"&amp;TEXT(C80,"0.00")&amp;"/kg and ₹"&amp;TEXT(C82,"0.00")&amp;"/kg earns a "&amp;TEXT(C81,"0%")&amp;" margin. At ₹"&amp;TEXT(C78,"0")&amp;"/kg we make ₹"&amp;TEXT(C84,"#,##0.0")&amp;" L a year. Every ₹1/kg higher price adds ₹"&amp;TEXT(C10*1000*(1-C34)/100000,"#,##0")&amp;" L a year."</f>
+        <v>We put in ₹351 L and sell 10,800 t a year. Break-even is ₹26.86/kg and ₹29.98/kg earns a 10% margin. At ₹28/kg we make ₹118.1 L a year. Every ₹1/kg higher price adds ₹104 L a year.</v>
+      </c>
+      <c r="C86" s="16"/>
+      <c r="D86" s="16"/>
+      <c r="E86" s="16"/>
+      <c r="F86" s="16"/>
+      <c r="G86" s="16"/>
+      <c r="H86" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="B17:H17"/>
-    <mergeCell ref="B84:H84"/>
+    <mergeCell ref="B19:H19"/>
+    <mergeCell ref="B86:H86"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3024,18 +3089,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="31" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="32" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="B3" s="32" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="C3" s="32" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3043,10 +3108,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="33" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="C4" s="33" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3054,10 +3119,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3065,10 +3130,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="33" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3076,10 +3141,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="33" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3087,10 +3152,10 @@
         <v>5</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3098,10 +3163,10 @@
         <v>6</v>
       </c>
       <c r="B9" s="33" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="C9" s="33" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3109,10 +3174,10 @@
         <v>7</v>
       </c>
       <c r="B10" s="33" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="C10" s="33" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3120,10 +3185,10 @@
         <v>8</v>
       </c>
       <c r="B11" s="33" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3131,10 +3196,10 @@
         <v>9</v>
       </c>
       <c r="B12" s="33" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="C12" s="33" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3142,10 +3207,10 @@
         <v>10</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
   </sheetData>

</xml_diff>